<commit_message>
Data sync: PhraseList +50 phrases, en audio for rows 14/183, sw v56
Source: updated PhraseList.xlsx + new English recordings for
"How are you today?" (Excel row 14) and "It's up to you." (row 183).
sync-updated-audio.mjs extended to also process the en/ folder; canonical
archive moved to repo-root audio-未压缩-原版/. oralPhrases.js now has 195
phrases (up from 145).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/update_data_folder/PhraseList.xlsx
+++ b/update_data_folder/PhraseList.xlsx
@@ -2,11 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet name="口语" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="物件记录" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -21,6 +25,7 @@
     </font>
     <font>
       <name val="Helvetica"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
     </font>
@@ -31,29 +36,34 @@
     </font>
     <font>
       <name val="Helvetica"/>
-      <color rgb="001F1F1F"/>
+      <family val="2"/>
+      <color rgb="FF1F1F1F"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Helvetica"/>
+      <family val="2"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Helvetica"/>
+      <family val="2"/>
       <color indexed="8"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Helvetica Neue"/>
+      <family val="2"/>
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill/>
     </fill>
@@ -67,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFD700"/>
+        <fgColor rgb="FFFFD700"/>
       </patternFill>
     </fill>
     <fill>
@@ -92,27 +102,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADD8E6"/>
+        <fgColor rgb="FFADD8E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998"/>
+        <fgColor theme="7" tint="0.7999511703848384"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998"/>
+        <fgColor theme="7" tint="0.7999511703848384"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998"/>
+        <fgColor theme="7" tint="0.7999511703848384"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
@@ -127,32 +140,38 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADD8E6"/>
+        <fgColor rgb="FFADD8E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
+        <fgColor rgb="FFFFC000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00ADD8E6"/>
+        <fgColor rgb="FFADD8E6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC9E1FF"/>
+        <bgColor rgb="FFC9E1FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -163,7 +182,13 @@
     </fill>
   </fills>
   <borders count="2">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left style="thin">
         <color auto="1"/>
@@ -177,6 +202,7 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -275,9 +301,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="16" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -301,10 +324,12 @@
     <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -518,6 +543,8 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -536,13 +563,13 @@
     <col width="7.1640625" customWidth="1" style="2" min="4" max="4"/>
     <col width="33" customWidth="1" style="6" min="5" max="5"/>
     <col width="24.33203125" customWidth="1" style="16" min="6" max="6"/>
-    <col width="11.5" customWidth="1" style="6" min="7" max="7"/>
+    <col width="32.1640625" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
     <col width="68.6640625" customWidth="1" style="6" min="8" max="8"/>
     <col width="113.83203125" customWidth="1" style="6" min="9" max="9"/>
     <col width="25.33203125" customWidth="1" style="6" min="10" max="10"/>
     <col width="91" customWidth="1" style="6" min="11" max="11"/>
-    <col width="10.83203125" customWidth="1" style="2" min="12" max="87"/>
-    <col width="10.83203125" customWidth="1" style="2" min="88" max="16384"/>
+    <col width="10.83203125" customWidth="1" style="2" min="12" max="88"/>
+    <col width="10.83203125" customWidth="1" style="2" min="89" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="1">
@@ -743,10 +770,10 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>zǎoshang hǎo</t>
-        </is>
-      </c>
-      <c r="H4" s="37" t="inlineStr">
+          <t>zǎoshànghǎo</t>
+        </is>
+      </c>
+      <c r="H4" s="36" t="inlineStr">
         <is>
           <t>窗帘懒洋洋地拉开，打了个哈欠说：“早上好呀，小太阳。”</t>
         </is>
@@ -911,7 +938,7 @@
           <t>duìbuqǐ</t>
         </is>
       </c>
-      <c r="H7" s="37" t="inlineStr">
+      <c r="H7" s="36" t="inlineStr">
         <is>
           <t>橡皮又擦掉一处小错误，叹了口气：“对不起啊，有我护着你呢。”</t>
         </is>
@@ -1018,7 +1045,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>shì de</t>
+          <t>shìde</t>
         </is>
       </c>
       <c r="H9" s="21" t="inlineStr">
@@ -1081,7 +1108,7 @@
           <t>红绿灯一下子变红了：“不行，你得等等。”</t>
         </is>
       </c>
-      <c r="I10" s="42" t="inlineStr">
+      <c r="I10" s="41" t="inlineStr">
         <is>
           <t>だめ</t>
         </is>
@@ -1126,9 +1153,9 @@
           <t>不好意思</t>
         </is>
       </c>
-      <c r="G11" s="46" t="inlineStr">
-        <is>
-          <t>bù hǎoyìsi</t>
+      <c r="G11" s="45" t="inlineStr">
+        <is>
+          <t>bùhǎoyìsi</t>
         </is>
       </c>
       <c r="H11" s="21" t="inlineStr">
@@ -1181,6 +1208,11 @@
           <t>不客气</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>bù kèqi</t>
+        </is>
+      </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
           <t>石头绊你一跤，咧嘴一笑：“不客气哦。”</t>
@@ -1191,7 +1223,7 @@
           <t>どういたしまして</t>
         </is>
       </c>
-      <c r="J12" s="45" t="inlineStr">
+      <c r="J12" s="44" t="inlineStr">
         <is>
           <t>dō itashimashite</t>
         </is>
@@ -1231,6 +1263,11 @@
           <t>很高兴认识你</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>hěn gāoxìng rènshi nǐ</t>
+        </is>
+      </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
           <t>胶水紧紧抱住你：“很高兴认识你——我再也不撒手啦。”</t>
@@ -1277,6 +1314,11 @@
           <t>你今天怎么样？</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>nǐ jīntiān zěnmeyàng</t>
+        </is>
+      </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
           <t>镜子每天早上看见你的脸，就问：“你今天怎么样？”</t>
@@ -1327,6 +1369,11 @@
           <t>我不明白</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>wǒ bù míngbai</t>
+        </is>
+      </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
           <t>计算器盯着算式一脸懵：“我不明白。”</t>
@@ -1377,6 +1424,11 @@
           <t>救命</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>jiùmìng</t>
+        </is>
+      </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
           <t>纽扣只剩一根线吊着，大喊：“救命啊！”</t>
@@ -1392,7 +1444,7 @@
           <t>tasukete</t>
         </is>
       </c>
-      <c r="K16" s="44" t="inlineStr">
+      <c r="K16" s="43" t="inlineStr">
         <is>
           <t>ボタンは糸一本でぶらーん。「助けて〜！」</t>
         </is>
@@ -1427,6 +1479,11 @@
           <t>嘿！</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>hēi</t>
+        </is>
+      </c>
       <c r="H17" s="21" t="inlineStr">
         <is>
           <t>弹窗广告蹦到屏幕上大喊：“嘿！快看我！”</t>
@@ -1477,6 +1534,11 @@
           <t>最近怎么样？</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>zuìjìn zěnmeyàng</t>
+        </is>
+      </c>
       <c r="H18" s="21" t="inlineStr">
         <is>
           <t>手机嗡嗡一震亮起来：“最近怎么样？”</t>
@@ -1527,7 +1589,12 @@
           <t>好久不见</t>
         </is>
       </c>
-      <c r="H19" s="38" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>hǎojiǔ bú jiàn</t>
+        </is>
+      </c>
+      <c r="H19" s="37" t="inlineStr">
         <is>
           <t>大衣从衣柜里被翻出来，咧嘴一笑：“好久不见！”</t>
         </is>
@@ -1577,7 +1644,12 @@
           <t>你最近过得怎么样？</t>
         </is>
       </c>
-      <c r="H20" s="37" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>nǐ zuìjìn guò de zěnmeyàng</t>
+        </is>
+      </c>
+      <c r="H20" s="36" t="inlineStr">
         <is>
           <t>洒水壶找到蔫蔫的小盆栽：“你最近过得怎么样？”</t>
         </is>
@@ -1627,6 +1699,11 @@
           <t>我挺好的，谢谢</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>wǒ tǐng hǎo de xièxie</t>
+        </is>
+      </c>
       <c r="H21" s="21" t="inlineStr">
         <is>
           <t>太阳能板美美地晒着太阳，笑着说：“我挺好的，谢谢！”</t>
@@ -1682,7 +1759,7 @@
           <t>hái xíng</t>
         </is>
       </c>
-      <c r="H22" s="37" t="inlineStr">
+      <c r="H22" s="36" t="inlineStr">
         <is>
           <t>二手沙发搬进客厅，耸耸肩说：“还行嘛。”</t>
         </is>
@@ -1734,7 +1811,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>lǎoyàngzi</t>
+          <t>lǎo yàngzi</t>
         </is>
       </c>
       <c r="H23" s="21" t="inlineStr">
@@ -1862,7 +1939,7 @@
           <t>mata ato de</t>
         </is>
       </c>
-      <c r="K25" s="44" t="inlineStr">
+      <c r="K25" s="43" t="inlineStr">
         <is>
           <t>ブーメラン、ひゅーんと飛んでいって、「またあとで！」</t>
         </is>
@@ -1917,7 +1994,7 @@
           <t>mata ashita</t>
         </is>
       </c>
-      <c r="K26" s="44" t="inlineStr">
+      <c r="K26" s="43" t="inlineStr">
         <is>
           <t>お日さま、地平線にゆうらり沈んで、手をふって、「また明日！」</t>
         </is>
@@ -2007,7 +2084,7 @@
           <t>我得走了</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G28" s="47" t="inlineStr">
         <is>
           <t>wǒ děi zǒu le</t>
         </is>
@@ -2122,7 +2199,7 @@
           <t>jiàndào nǐ zhēn gāoxìng</t>
         </is>
       </c>
-      <c r="H30" s="37" t="inlineStr">
+      <c r="H30" s="36" t="inlineStr">
         <is>
           <t>灯塔朝路过的船眨眨眼，喊道：“见到你真高兴！”</t>
         </is>
@@ -2242,7 +2319,7 @@
           <t>おかえりなさい</t>
         </is>
       </c>
-      <c r="J32" s="45" t="inlineStr">
+      <c r="J32" s="44" t="inlineStr">
         <is>
           <t>okaeri nasai</t>
         </is>
@@ -2282,7 +2359,7 @@
           <t>你看起来真棒</t>
         </is>
       </c>
-      <c r="G33" s="46" t="inlineStr">
+      <c r="G33" s="45" t="inlineStr">
         <is>
           <t>nǐ kàn qǐlái zhēn bàng</t>
         </is>
@@ -2339,7 +2416,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>hēi, zuìjìn zěnmeyàng?</t>
+          <t>hēi，zuìjìn zěnmeyàng？</t>
         </is>
       </c>
       <c r="H34" s="21" t="inlineStr">
@@ -2449,7 +2526,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>zhēnshì tài gǎnxiè le</t>
+          <t>zhēn shì tài gǎnxiè le</t>
         </is>
       </c>
       <c r="H36" s="21" t="inlineStr">
@@ -2502,7 +2579,7 @@
           <t>我真的很感动</t>
         </is>
       </c>
-      <c r="G37" s="46" t="inlineStr">
+      <c r="G37" s="45" t="inlineStr">
         <is>
           <t>wǒ zhēn de hěn gǎndòng</t>
         </is>
@@ -2559,7 +2636,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>nǐ zhēnshì bāng le wǒ dàmáng</t>
+          <t>nǐ zhēn shì bāng le wǒ dà máng</t>
         </is>
       </c>
       <c r="H38" s="24" t="inlineStr">
@@ -2577,7 +2654,7 @@
           <t>hontō ni tasukarimashita</t>
         </is>
       </c>
-      <c r="K38" s="44" t="inlineStr">
+      <c r="K38" s="43" t="inlineStr">
         <is>
           <t>おぼれかけのビーチサンダル、浮き輪を見て泣きさけぶ。「本当に助かりました！」</t>
         </is>
@@ -2612,7 +2689,7 @@
           <t>我欠你一个人情</t>
         </is>
       </c>
-      <c r="G39" s="46" t="inlineStr">
+      <c r="G39" s="45" t="inlineStr">
         <is>
           <t>wǒ qiàn nǐ yí gè rénqíng</t>
         </is>
@@ -2667,7 +2744,7 @@
           <t>没事儿</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="47" t="inlineStr">
         <is>
           <t>méishìr</t>
         </is>
@@ -2792,7 +2869,7 @@
           <t>いつでもどうぞ</t>
         </is>
       </c>
-      <c r="J42" s="45" t="inlineStr">
+      <c r="J42" s="44" t="inlineStr">
         <is>
           <t>itsu demo dōzo</t>
         </is>
@@ -2842,7 +2919,7 @@
           <t>自动纠错把你的名字改成了“鸭子”，还说：“我的错。”</t>
         </is>
       </c>
-      <c r="I43" s="43" t="inlineStr">
+      <c r="I43" s="42" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;私&lt;rt&gt;わたし&lt;/rt&gt;&lt;/ruby&gt;のミスです</t>
         </is>
@@ -2947,7 +3024,7 @@
           <t>zhè shì guài wǒ</t>
         </is>
       </c>
-      <c r="H45" s="37" t="inlineStr">
+      <c r="H45" s="36" t="inlineStr">
         <is>
           <t>小心地滑的牌子扑通倒下来把你绊了一跤，叹口气说：“这事怪我。”</t>
         </is>
@@ -2962,7 +3039,7 @@
           <t>watashi no sei deshita</t>
         </is>
       </c>
-      <c r="K45" s="44" t="inlineStr">
+      <c r="K45" s="43" t="inlineStr">
         <is>
           <t>『足もと注意』の看板がぱたんと倒れて、きみをつまずかせ、はあ。「私のせいでした」</t>
         </is>
@@ -3054,7 +3131,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>xiàcì bú huì le</t>
+          <t>xià cì bú huì le</t>
         </is>
       </c>
       <c r="H47" s="16" t="inlineStr">
@@ -3117,7 +3194,7 @@
           <t>购物袋都快撑破了，还笑着说：“完全没问题！”</t>
         </is>
       </c>
-      <c r="I48" s="42" t="inlineStr">
+      <c r="I48" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;全然問題&lt;rt&gt;ぜんぜんもんだい&lt;/rt&gt;&lt;/ruby&gt;ありません</t>
         </is>
@@ -3164,10 +3241,10 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>xièxie nǐ wèi wǒ zuò de yíqiè</t>
-        </is>
-      </c>
-      <c r="H49" s="39" t="inlineStr">
+          <t>xièxie nǐ wèi wǒ zuò de yīqiè</t>
+        </is>
+      </c>
+      <c r="H49" s="38" t="inlineStr">
         <is>
           <t>生日蜡烛坐在蛋糕上，笑眯眯地说：“谢谢你为我做的一切。”</t>
         </is>
@@ -3217,7 +3294,7 @@
           <t>真是欠你个大人情</t>
         </is>
       </c>
-      <c r="G50" s="46" t="inlineStr">
+      <c r="G50" s="45" t="inlineStr">
         <is>
           <t>zhēn shì qiàn nǐ gè dà rénqíng</t>
         </is>
@@ -3442,12 +3519,12 @@
           <t>nǐ shuō de duì</t>
         </is>
       </c>
-      <c r="H54" s="37" t="inlineStr">
+      <c r="H54" s="36" t="inlineStr">
         <is>
           <t>导航重新规划了三次，最后叹口气：“你说得对。”</t>
         </is>
       </c>
-      <c r="I54" s="42" t="inlineStr">
+      <c r="I54" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;確&lt;rt&gt;たし&lt;/rt&gt;&lt;/ruby&gt;かにそうです</t>
         </is>
@@ -3492,9 +3569,9 @@
           <t>我这边也一样</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>wǒ zhèbiān yě yíyàng</t>
+      <c r="G55" s="47" t="inlineStr">
+        <is>
+          <t>wǒ zhè biān yě yíyàng</t>
         </is>
       </c>
       <c r="H55" s="21" t="inlineStr">
@@ -3567,7 +3644,7 @@
           <t>watashi mo desu</t>
         </is>
       </c>
-      <c r="K56" s="44" t="inlineStr">
+      <c r="K56" s="43" t="inlineStr">
         <is>
           <t>影は猫ちゃんの動きをそっくりまねして、大きな声で「私もです！」</t>
         </is>
@@ -3607,12 +3684,12 @@
           <t>xíng ba</t>
         </is>
       </c>
-      <c r="H57" s="38" t="inlineStr">
+      <c r="H57" s="37" t="inlineStr">
         <is>
           <t>硬币落地，反面朝上，叹了口气：“行吧。”</t>
         </is>
       </c>
-      <c r="I57" s="43" t="inlineStr">
+      <c r="I57" s="42" t="inlineStr">
         <is>
           <t>まあ、しかたないですね</t>
         </is>
@@ -3712,12 +3789,12 @@
           <t>这我可不好说</t>
         </is>
       </c>
-      <c r="G59" s="46" t="inlineStr">
+      <c r="G59" s="45" t="inlineStr">
         <is>
           <t>zhè wǒ kě bù hǎo shuō</t>
         </is>
       </c>
-      <c r="H59" s="38" t="inlineStr">
+      <c r="H59" s="37" t="inlineStr">
         <is>
           <t>天气App盯着云朵嘟囔：“这我可不好说。”</t>
         </is>
@@ -3769,7 +3846,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>wǒ bú zhème juéde</t>
+          <t>wǒ bù zhème juéde</t>
         </is>
       </c>
       <c r="H60" s="21" t="inlineStr">
@@ -3822,7 +3899,7 @@
           <t>这说不通啊</t>
         </is>
       </c>
-      <c r="G61" s="46" t="inlineStr">
+      <c r="G61" s="47" t="inlineStr">
         <is>
           <t>zhè shuōbutōng a</t>
         </is>
@@ -3932,12 +4009,12 @@
           <t>还是算了</t>
         </is>
       </c>
-      <c r="G63" s="46" t="inlineStr">
+      <c r="G63" s="47" t="inlineStr">
         <is>
           <t>háishi suàn le</t>
         </is>
       </c>
-      <c r="H63" s="37" t="inlineStr">
+      <c r="H63" s="36" t="inlineStr">
         <is>
           <t>回收桶吐出一个塑料袋：“嗯……还是算了。”</t>
         </is>
@@ -3952,7 +4029,7 @@
           <t>yappari yamete okimasu</t>
         </is>
       </c>
-      <c r="K63" s="37" t="inlineStr">
+      <c r="K63" s="36" t="inlineStr">
         <is>
           <t>リサイクルボックス、ビニール袋をぺっと吐き出して、「やっぱりやめておきます」</t>
         </is>
@@ -3989,7 +4066,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>juéduì bù xíng</t>
+          <t>juéduì bùxíng</t>
         </is>
       </c>
       <c r="H64" s="21" t="inlineStr">
@@ -4042,12 +4119,12 @@
           <t>我累死了</t>
         </is>
       </c>
-      <c r="G65" s="46" t="inlineStr">
-        <is>
-          <t>wǒ lèisǐ le</t>
-        </is>
-      </c>
-      <c r="H65" s="37" t="inlineStr">
+      <c r="G65" s="45" t="inlineStr">
+        <is>
+          <t>wǒ lèi sǐ le</t>
+        </is>
+      </c>
+      <c r="H65" s="36" t="inlineStr">
         <is>
           <t>电池一闪一闪，嘟囔着：“我累死了。”</t>
         </is>
@@ -4097,12 +4174,12 @@
           <t>饿死我了</t>
         </is>
       </c>
-      <c r="G66" s="46" t="inlineStr">
-        <is>
-          <t>èsǐ wǒ le</t>
-        </is>
-      </c>
-      <c r="H66" s="37" t="inlineStr">
+      <c r="G66" s="45" t="inlineStr">
+        <is>
+          <t>è sǐ wǒ le</t>
+        </is>
+      </c>
+      <c r="H66" s="36" t="inlineStr">
         <is>
           <t>空冰箱打开门哭着喊：“饿死我了！”</t>
         </is>
@@ -4152,12 +4229,12 @@
           <t>冻死我了</t>
         </is>
       </c>
-      <c r="G67" s="46" t="inlineStr">
+      <c r="G67" s="45" t="inlineStr">
         <is>
           <t>dòng sǐ wǒ le</t>
         </is>
       </c>
-      <c r="H67" s="37" t="inlineStr">
+      <c r="H67" s="36" t="inlineStr">
         <is>
           <t>冰淇淋围上小围巾，嘟囔着：“冻死我了。”</t>
         </is>
@@ -4167,7 +4244,7 @@
           <t>&lt;ruby&gt;凍&lt;rt&gt;こご&lt;/rt&gt;&lt;/ruby&gt;えそうです</t>
         </is>
       </c>
-      <c r="J67" s="45" t="inlineStr">
+      <c r="J67" s="44" t="inlineStr">
         <is>
           <t>kogoesō desu</t>
         </is>
@@ -4207,12 +4284,12 @@
           <t>无聊死了</t>
         </is>
       </c>
-      <c r="G68" s="46" t="inlineStr">
+      <c r="G68" s="45" t="inlineStr">
         <is>
           <t>wúliáo sǐ le</t>
         </is>
       </c>
-      <c r="H68" s="37" t="inlineStr">
+      <c r="H68" s="36" t="inlineStr">
         <is>
           <t>木马哼哼着：“无聊死了，天天转圈圈。”</t>
         </is>
@@ -4227,7 +4304,7 @@
           <t>taikutsu de tamarimasen</t>
         </is>
       </c>
-      <c r="K68" s="44" t="inlineStr">
+      <c r="K68" s="43" t="inlineStr">
         <is>
           <t>メリーゴーランドの木馬がうめく。「退屈でたまりません。毎日おんなじところをぐるぐる」</t>
         </is>
@@ -4267,7 +4344,7 @@
           <t>wǒ yǒudiǎn jǐnzhāng</t>
         </is>
       </c>
-      <c r="H69" s="37" t="inlineStr">
+      <c r="H69" s="36" t="inlineStr">
         <is>
           <t>钢丝晃晃悠悠，小声说：“我有点紧张。”</t>
         </is>
@@ -4322,7 +4399,7 @@
           <t>wǒ tài jīdòng le</t>
         </is>
       </c>
-      <c r="H70" s="37" t="inlineStr">
+      <c r="H70" s="36" t="inlineStr">
         <is>
           <t>礼物盒摇来晃去，尖叫着：“我太激动了！”</t>
         </is>
@@ -4337,7 +4414,7 @@
           <t>sugoku wakuwaku shite imasu</t>
         </is>
       </c>
-      <c r="K70" s="44" t="inlineStr">
+      <c r="K70" s="43" t="inlineStr">
         <is>
           <t>プレゼントの箱がぶるぶるふるえて、「すごくワクワクしています！」</t>
         </is>
@@ -4372,7 +4449,7 @@
           <t>我今天心情不错</t>
         </is>
       </c>
-      <c r="G71" s="46" t="inlineStr">
+      <c r="G71" s="45" t="inlineStr">
         <is>
           <t>wǒ jīntiān xīnqíng búcuò</t>
         </is>
@@ -4447,7 +4524,7 @@
           <t>sonna kibun ja nai desu</t>
         </is>
       </c>
-      <c r="K72" s="44" t="inlineStr">
+      <c r="K72" s="43" t="inlineStr">
         <is>
           <t>プリンター、エラーランプをぴかぴか。「そんな気分じゃないです」とぶつぶつ。</t>
         </is>
@@ -4482,17 +4559,17 @@
           <t>这让我开心了一整天</t>
         </is>
       </c>
-      <c r="G73" s="46" t="inlineStr">
+      <c r="G73" s="45" t="inlineStr">
         <is>
           <t>zhè ràng wǒ kāixīn le yì zhěng tiān</t>
         </is>
       </c>
-      <c r="H73" s="37" t="inlineStr">
+      <c r="H73" s="36" t="inlineStr">
         <is>
           <t>日历翻到新的一页，笑得合不拢嘴：“这让我开心了一整天！”</t>
         </is>
       </c>
-      <c r="I73" s="42" t="inlineStr">
+      <c r="I73" s="41" t="inlineStr">
         <is>
           <t>おかげでいい&lt;ruby&gt;一日&lt;rt&gt;いちにち&lt;/rt&gt;&lt;/ruby&gt;になりました</t>
         </is>
@@ -4542,7 +4619,7 @@
           <t>xiào sǐ wǒ le</t>
         </is>
       </c>
-      <c r="H74" s="37" t="inlineStr">
+      <c r="H74" s="36" t="inlineStr">
         <is>
           <t>鸡毛掸子把自己挠得痒痒的，咯咯直叫：“笑死我了。”</t>
         </is>
@@ -4602,7 +4679,7 @@
           <t>小黄鸭被捏了一下，吱吱叫：“太好笑了！”</t>
         </is>
       </c>
-      <c r="I75" s="42" t="inlineStr">
+      <c r="I75" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;面白&lt;rt&gt;おもしろ&lt;/rt&gt;&lt;/ruby&gt;すぎます</t>
         </is>
@@ -4612,7 +4689,7 @@
           <t>omoshirosugimasu</t>
         </is>
       </c>
-      <c r="K75" s="44" t="inlineStr">
+      <c r="K75" s="43" t="inlineStr">
         <is>
           <t>アヒルさん、ぎゅっとつままれて、キュッ。「面白すぎます！」</t>
         </is>
@@ -4667,7 +4744,7 @@
           <t>tsurai desu ne</t>
         </is>
       </c>
-      <c r="K76" s="44" t="inlineStr">
+      <c r="K76" s="43" t="inlineStr">
         <is>
           <t>ばんそうこう、ぺりっと自分をはがして、ふぅ。「つらいですね」</t>
         </is>
@@ -4707,7 +4784,7 @@
           <t>zhēn fánrén</t>
         </is>
       </c>
-      <c r="H77" s="38" t="inlineStr">
+      <c r="H77" s="37" t="inlineStr">
         <is>
           <t>手机第十次嗡嗡响，没好气地哼一声：“真烦人。”</t>
         </is>
@@ -4812,7 +4889,7 @@
           <t>那真让我压力山大</t>
         </is>
       </c>
-      <c r="G79" s="46" t="inlineStr">
+      <c r="G79" s="47" t="inlineStr">
         <is>
           <t>nà zhēn ràng wǒ yālì shāndà</t>
         </is>
@@ -4822,7 +4899,7 @@
           <t>气球哆嗦地说：“那真让我压力山大。”</t>
         </is>
       </c>
-      <c r="I79" s="43" t="inlineStr">
+      <c r="I79" s="42" t="inlineStr">
         <is>
           <t>すごくストレスでした</t>
         </is>
@@ -4867,7 +4944,7 @@
           <t>总算松了一口气</t>
         </is>
       </c>
-      <c r="G80" s="46" t="inlineStr">
+      <c r="G80" s="45" t="inlineStr">
         <is>
           <t>zǒngsuàn sōng le yì kǒu qì</t>
         </is>
@@ -4977,6 +5054,11 @@
           <t>我想你了</t>
         </is>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>wǒ xiǎng nǐ le</t>
+        </is>
+      </c>
       <c r="H82" s="21" t="inlineStr">
         <is>
           <t>孤单小袜子盯着烘干机，小声说：“我想你了。”</t>
@@ -5027,6 +5109,11 @@
           <t>我真的受够了</t>
         </is>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>wǒ zhēn de shòugòu le</t>
+        </is>
+      </c>
       <c r="H83" s="21" t="inlineStr">
         <is>
           <t>打印机第三次卡纸了，咕哝着：“我真的受够了。”</t>
@@ -5077,7 +5164,12 @@
           <t>今天真是太棒了</t>
         </is>
       </c>
-      <c r="H84" s="37" t="inlineStr">
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>jīntiān zhēn shì tài bàng le</t>
+        </is>
+      </c>
+      <c r="H84" s="36" t="inlineStr">
         <is>
           <t>大热天，电风扇一开机就大喊：“今天真是太棒了！”</t>
         </is>
@@ -5092,7 +5184,7 @@
           <t>kyō wa saikō no ichinichi desu</t>
         </is>
       </c>
-      <c r="K84" s="44" t="inlineStr">
+      <c r="K84" s="43" t="inlineStr">
         <is>
           <t>むわっと暑い日、スイッチの入った扇風機、「今日は最高の一日です！」と大さけび。</t>
         </is>
@@ -5127,6 +5219,11 @@
           <t>要不要一起出来玩？</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>yào bu yào yìqǐ chūlái wán</t>
+        </is>
+      </c>
       <c r="H85" s="21" t="inlineStr">
         <is>
           <t>小蝙蝠倒挂着，冲大家喊：“要不要一起出来玩？”</t>
@@ -5177,7 +5274,12 @@
           <t>一起去喝杯咖啡吧</t>
         </is>
       </c>
-      <c r="H86" s="38" t="inlineStr">
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>yìqǐ qù hē bēi kāfēi ba</t>
+        </is>
+      </c>
+      <c r="H86" s="37" t="inlineStr">
         <is>
           <t>水壶哼了一声：“一起去喝杯咖啡吧，我天天煮都煮烦啦。”</t>
         </is>
@@ -5227,7 +5329,12 @@
           <t>下次再聚啊</t>
         </is>
       </c>
-      <c r="H87" s="37" t="inlineStr">
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>xià cì zài jù a</t>
+        </is>
+      </c>
+      <c r="H87" s="36" t="inlineStr">
         <is>
           <t>过山车缓缓滑回站台：“下次再聚啊！”</t>
         </is>
@@ -5242,7 +5349,7 @@
           <t>mata atsumarimashō</t>
         </is>
       </c>
-      <c r="K87" s="44" t="inlineStr">
+      <c r="K87" s="43" t="inlineStr">
         <is>
           <t>ジェットコースター、乗り場にするすると戻ってきて、「また集まりましょう！」</t>
         </is>
@@ -5277,6 +5384,11 @@
           <t>你应该试试</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>nǐ yīnggāi shìshi</t>
+        </is>
+      </c>
       <c r="H88" s="21" t="inlineStr">
         <is>
           <t>辣椒酱滑到你盘子边，咧嘴一笑：“你应该试试。”</t>
@@ -5327,7 +5439,12 @@
           <t>我们一起去吧？</t>
         </is>
       </c>
-      <c r="H89" s="37" t="inlineStr">
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>wǒmen yìqǐ qù ba</t>
+        </is>
+      </c>
+      <c r="H89" s="36" t="inlineStr">
         <is>
           <t>左鞋碰碰右鞋：“我们一起去吧？”</t>
         </is>
@@ -5377,6 +5494,11 @@
           <t>这周末怎么样？</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>zhè zhōumò zěnmeyàng</t>
+        </is>
+      </c>
       <c r="H90" s="21" t="inlineStr">
         <is>
           <t>洗衣机瞟了眼那堆脏衣服，叹气说：“这周末怎么样？”</t>
@@ -5427,7 +5549,12 @@
           <t>咱们平分吧</t>
         </is>
       </c>
-      <c r="H91" s="40" t="inlineStr">
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>zánmen píngfēn ba</t>
+        </is>
+      </c>
+      <c r="H91" s="39" t="inlineStr">
         <is>
           <t>一只筷子悄悄对另一只说：“咱们平分吧。”</t>
         </is>
@@ -5477,6 +5604,11 @@
           <t>我请你</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>wǒ qǐng nǐ</t>
+        </is>
+      </c>
       <c r="H92" s="21" t="inlineStr">
         <is>
           <t>自动售货机掉出一包零食：“我请你！”</t>
@@ -5527,7 +5659,12 @@
           <t>我请客</t>
         </is>
       </c>
-      <c r="H93" s="41" t="inlineStr">
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>wǒ qǐngkè</t>
+        </is>
+      </c>
+      <c r="H93" s="40" t="inlineStr">
         <is>
           <t>苹果树啪地往你头上扔下一颗果子，欢快地说：“我请客！”</t>
         </is>
@@ -5577,6 +5714,11 @@
           <t>你待会儿有空吗？</t>
         </is>
       </c>
+      <c r="G94" s="47" t="inlineStr">
+        <is>
+          <t>nǐ dāihuìr yǒu kòng ma?</t>
+        </is>
+      </c>
       <c r="H94" s="21" t="inlineStr">
         <is>
           <t>风筝拽了拽线，叹气问：“你待会儿有空吗？”</t>
@@ -5627,12 +5769,17 @@
           <t>过来吧</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>guòlái ba</t>
+        </is>
+      </c>
       <c r="H95" s="21" t="inlineStr">
         <is>
           <t>磁铁冲着冰箱大喊：“过来吧！我够不着你呀！”</t>
         </is>
       </c>
-      <c r="I95" s="42" t="inlineStr">
+      <c r="I95" s="41" t="inlineStr">
         <is>
           <t>こっちにおいでよ</t>
         </is>
@@ -5677,6 +5824,11 @@
           <t>有空跟我说一声</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>yǒu kòng gēn wǒ shuō yì shēng</t>
+        </is>
+      </c>
       <c r="H96" s="21" t="inlineStr">
         <is>
           <t>日历哗啦啦翻着页：“有空跟我说一声哦。”</t>
@@ -5727,6 +5879,11 @@
           <t>千万别错过</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>qiānwàn bié cuòguò</t>
+        </is>
+      </c>
       <c r="H97" s="21" t="inlineStr">
         <is>
           <t>流星嗖地划过天空，大喊：“千万别错过！”</t>
@@ -5742,7 +5899,7 @@
           <t>ominogashi naku</t>
         </is>
       </c>
-      <c r="K97" s="44" t="inlineStr">
+      <c r="K97" s="43" t="inlineStr">
         <is>
           <t>流れ星、空をシュッとかけぬけて、「お見逃しなく！」と叫ぶ。</t>
         </is>
@@ -5777,6 +5934,11 @@
           <t>你会来吧？</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>nǐ huì lái ba</t>
+        </is>
+      </c>
       <c r="H98" s="21" t="inlineStr">
         <is>
           <t>鱼钩沉进水里，小声问鱼儿：“你会来吧？”</t>
@@ -5827,6 +5989,11 @@
           <t>我能要这个吗？</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>wǒ néng yào zhège ma</t>
+        </is>
+      </c>
       <c r="H99" s="22" t="inlineStr">
         <is>
           <t>小猪存钱罐把鼻子贴在橱窗上，小声问：“我能要这个吗？”</t>
@@ -5842,7 +6009,7 @@
           <t>kore, katte mo ii desu ka?</t>
         </is>
       </c>
-      <c r="K99" s="44" t="inlineStr">
+      <c r="K99" s="43" t="inlineStr">
         <is>
           <t>ぶたの貯金箱、ショーウィンドウに鼻をぺたり。「これ、買ってもいいですか？」</t>
         </is>
@@ -5877,6 +6044,11 @@
           <t>这个多少钱？</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>zhège duōshao qián</t>
+        </is>
+      </c>
       <c r="H100" s="21" t="inlineStr">
         <is>
           <t>古董花瓶拎起价签，眯眼瞧：“这个多少钱？”</t>
@@ -5927,6 +6099,11 @@
           <t>这个有别的尺码吗？</t>
         </is>
       </c>
+      <c r="G101" s="45" t="inlineStr">
+        <is>
+          <t>zhège yǒu bié de chǐmǎ ma</t>
+        </is>
+      </c>
       <c r="H101" s="21" t="inlineStr">
         <is>
           <t>小金鱼盯着自己的小鱼缸，嘟囔着：“这个有别的尺码吗？”</t>
@@ -5977,6 +6154,11 @@
           <t>我能试穿一下吗</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>wǒ néng shìchuān yīxià ma</t>
+        </is>
+      </c>
       <c r="H102" s="22" t="inlineStr">
         <is>
           <t>寄居蟹捡起一个新壳，咧嘴一笑：“我能试穿一下吗？”</t>
@@ -6027,6 +6209,11 @@
           <t>就要这个了</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>jiù yào zhège le</t>
+        </is>
+      </c>
       <c r="H103" s="21" t="inlineStr">
         <is>
           <t>龙卷风卷过小镇，耸耸肩：“就要这个了。”</t>
@@ -6077,6 +6264,11 @@
           <t>随便看看，谢谢</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>suíbiàn kànkan，xièxie</t>
+        </is>
+      </c>
       <c r="H104" s="21" t="inlineStr">
         <is>
           <t>猫头鹰走进小店，眨眨眼：“随便看看，谢谢。”</t>
@@ -6127,6 +6319,11 @@
           <t>有更便宜的吗？</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>yǒu gèng piányí de ma</t>
+        </is>
+      </c>
       <c r="H105" s="21" t="inlineStr">
         <is>
           <t>小硬币皱着眉看价签，嘟囔：“有更便宜的吗？”</t>
@@ -6177,6 +6374,11 @@
           <t>能刷卡吗？</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>néng shuākǎ ma</t>
+        </is>
+      </c>
       <c r="H106" s="21" t="inlineStr">
         <is>
           <t>信用卡蹦上柜台问：“能刷卡吗？”</t>
@@ -6227,6 +6429,11 @@
           <t>不用找了</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>bùyòng zhǎo le</t>
+        </is>
+      </c>
       <c r="H107" s="21" t="inlineStr">
         <is>
           <t>自动售货机吞下你的硬币，咧嘴一笑：“不用找了。”</t>
@@ -6277,7 +6484,12 @@
           <t>能给我个袋子吗？</t>
         </is>
       </c>
-      <c r="H108" s="37" t="inlineStr">
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>néng gěi wǒ gè dàizi ma</t>
+        </is>
+      </c>
+      <c r="H108" s="36" t="inlineStr">
         <is>
           <t>茶叶东张西望，小声问：“能给我个袋子吗？”</t>
         </is>
@@ -6292,7 +6504,7 @@
           <t>fukuro o moraemasu ka?</t>
         </is>
       </c>
-      <c r="K108" s="44" t="inlineStr">
+      <c r="K108" s="43" t="inlineStr">
         <is>
           <t>茶葉はきょろきょろ見まわして、こっそり「袋をもらえますか？」</t>
         </is>
@@ -6327,6 +6539,11 @@
           <t>我要一样的</t>
         </is>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>wǒ yào yīyàng de</t>
+        </is>
+      </c>
       <c r="H109" s="21" t="inlineStr">
         <is>
           <t>影子看你点完餐，点点头说：“我要一样的。”</t>
@@ -6377,6 +6594,11 @@
           <t>可以打包吗？</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>kěyǐ dǎbāo ma</t>
+        </is>
+      </c>
       <c r="H110" s="21" t="inlineStr">
         <is>
           <t>饭盒朝服务员挥挥手：“可以打包吗？”</t>
@@ -6427,7 +6649,12 @@
           <t>有什么推荐的吗？</t>
         </is>
       </c>
-      <c r="H111" s="37" t="inlineStr">
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>yǒu shénme tuījiàn de ma</t>
+        </is>
+      </c>
+      <c r="H111" s="36" t="inlineStr">
         <is>
           <t>神奇八号球摇了摇身子：“有什么推荐的吗？”</t>
         </is>
@@ -6487,7 +6714,7 @@
           <t>钱包哼哼唧唧，小声说：“麻烦买单。”</t>
         </is>
       </c>
-      <c r="I112" s="43" t="inlineStr">
+      <c r="I112" s="42" t="inlineStr">
         <is>
           <t>お&lt;ruby&gt;会計&lt;rt&gt;かいけい&lt;/rt&gt;&lt;/ruby&gt;お&lt;ruby&gt;願&lt;rt&gt;ねが&lt;/rt&gt;&lt;/ruby&gt;いします</t>
         </is>
@@ -6497,7 +6724,7 @@
           <t>okaikei onegai shimasu</t>
         </is>
       </c>
-      <c r="K112" s="44" t="inlineStr">
+      <c r="K112" s="43" t="inlineStr">
         <is>
           <t>お財布がううっとうめいて、小さな声で。「お会計お願いします」</t>
         </is>
@@ -6534,10 +6761,10 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>zhège là ma？</t>
-        </is>
-      </c>
-      <c r="H113" s="37" t="inlineStr">
+          <t>zhège là ma</t>
+        </is>
+      </c>
+      <c r="H113" s="36" t="inlineStr">
         <is>
           <t>灭火器盯着辣椒酱，咽了咽口水问：“这个辣吗？”</t>
         </is>
@@ -6589,7 +6816,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>néng zài xù yì bēi ma？</t>
+          <t>néng zài xù yī bēi ma</t>
         </is>
       </c>
       <c r="H114" s="21" t="inlineStr">
@@ -6644,7 +6871,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>xǐshǒujiān zài nǎlǐ？</t>
+          <t>xǐshǒujiān zài nǎlǐ</t>
         </is>
       </c>
       <c r="H115" s="21" t="inlineStr">
@@ -6699,7 +6926,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>chēzhàn zěnme zǒu？</t>
+          <t>chēzhàn zěnme zǒu</t>
         </is>
       </c>
       <c r="H116" s="16" t="inlineStr">
@@ -6717,7 +6944,7 @@
           <t>eki ni wa dō ikeba ii desu ka?</t>
         </is>
       </c>
-      <c r="K116" s="44" t="inlineStr">
+      <c r="K116" s="43" t="inlineStr">
         <is>
           <t>きっぷが風にひらひら、大きな声で。「駅にはどう行けばいいですか？」</t>
         </is>
@@ -6754,7 +6981,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>lí zhèlǐ yuǎn ma？</t>
+          <t>lí zhèlǐ yuǎn ma</t>
         </is>
       </c>
       <c r="H117" s="21" t="inlineStr">
@@ -6807,9 +7034,9 @@
           <t>能在地图上指给我看吗？</t>
         </is>
       </c>
-      <c r="G118" s="46" t="inlineStr">
-        <is>
-          <t>néng zài dìtú shàng zhǐ gěi wǒ kàn ma?</t>
+      <c r="G118" s="45" t="inlineStr">
+        <is>
+          <t>néng zài dìtú shàng zhǐ gěi wǒ kàn ma</t>
         </is>
       </c>
       <c r="H118" s="21" t="inlineStr">
@@ -6919,7 +7146,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>yìzhí wǎng qián zǒu</t>
+          <t>yīzhí wǎng qián zǒu</t>
         </is>
       </c>
       <c r="H120" s="21" t="inlineStr">
@@ -6937,7 +7164,7 @@
           <t>massugu susunde kudasai</t>
         </is>
       </c>
-      <c r="K120" s="44" t="inlineStr">
+      <c r="K120" s="43" t="inlineStr">
         <is>
           <t>ナビくん、途中でぴたっと止まって、もごもご。「えーっと…まっすぐ進んでください？」</t>
         </is>
@@ -6977,7 +7204,7 @@
           <t>jiù zài fùjìn</t>
         </is>
       </c>
-      <c r="H121" s="39" t="inlineStr">
+      <c r="H121" s="38" t="inlineStr">
         <is>
           <t>迷宫偷偷笑着小声说：“就在附近，拐个弯就到。”</t>
         </is>
@@ -7029,7 +7256,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>yìyǎn jiù néng kànjiàn</t>
+          <t>yì yǎn jiù néng kànjiàn</t>
         </is>
       </c>
       <c r="H122" s="21" t="inlineStr">
@@ -7084,7 +7311,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>wǒ zǒu de fāngxiàng duì ma？</t>
+          <t>wǒ zǒu de fāngxiàng duì ma</t>
         </is>
       </c>
       <c r="H123" s="22" t="inlineStr">
@@ -7194,7 +7421,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>bàoqiàn，nǐ gāngcái shuō shénme？</t>
+          <t>bàoqiàn，nǐ gāngcái shuō shénme</t>
         </is>
       </c>
       <c r="H125" s="21" t="inlineStr">
@@ -7202,12 +7429,12 @@
           <t>助听器嗡嗡响：“抱歉，你刚才说什么？”</t>
         </is>
       </c>
-      <c r="I125" s="43" t="inlineStr">
+      <c r="I125" s="42" t="inlineStr">
         <is>
           <t>すみません&lt;ruby&gt;今&lt;rt&gt;いま&lt;/rt&gt;&lt;/ruby&gt;&lt;ruby&gt;何&lt;rt&gt;なん&lt;/rt&gt;&lt;/ruby&gt;て&lt;ruby&gt;言&lt;rt&gt;い&lt;/rt&gt;&lt;/ruby&gt;いましたか？</t>
         </is>
       </c>
-      <c r="J125" s="45" t="inlineStr">
+      <c r="J125" s="44" t="inlineStr">
         <is>
           <t>sumimasen ima nan te iimashita ka?</t>
         </is>
@@ -7249,7 +7476,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>néng zài shuō yíbiàn ma？</t>
+          <t>néng zài shuō yíbiàn ma</t>
         </is>
       </c>
       <c r="H126" s="21" t="inlineStr">
@@ -7262,7 +7489,7 @@
           <t>もう&lt;ruby&gt;一度&lt;rt&gt;いちど&lt;/rt&gt;&lt;/ruby&gt;&lt;ruby&gt;言&lt;rt&gt;い&lt;/rt&gt;&lt;/ruby&gt;ってもらえますか？</t>
         </is>
       </c>
-      <c r="J126" s="45" t="inlineStr">
+      <c r="J126" s="44" t="inlineStr">
         <is>
           <t>mō ichido itte moraemasu ka?</t>
         </is>
@@ -7304,7 +7531,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>néng shuō màn yìdiǎn ma？</t>
+          <t>néng shuō màn yìdiǎn ma</t>
         </is>
       </c>
       <c r="H127" s="21" t="inlineStr">
@@ -7359,10 +7586,10 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>nà shì shénme yìsi？</t>
-        </is>
-      </c>
-      <c r="H128" s="37" t="inlineStr">
+          <t>nà shì shénme yìsi</t>
+        </is>
+      </c>
+      <c r="H128" s="36" t="inlineStr">
         <is>
           <t>字典哗啦啦翻着自己的书页，气呼呼地问：“那是什么意思？”</t>
         </is>
@@ -7372,7 +7599,7 @@
           <t>それはどういう&lt;ruby&gt;意味&lt;rt&gt;いみ&lt;/rt&gt;&lt;/ruby&gt;ですか？</t>
         </is>
       </c>
-      <c r="J128" s="45" t="inlineStr">
+      <c r="J128" s="44" t="inlineStr">
         <is>
           <t>sore wa dō iu imi desu ka?</t>
         </is>
@@ -7414,7 +7641,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>zhège zěnme pīn？</t>
+          <t>zhège zěnme pīn</t>
         </is>
       </c>
       <c r="H129" s="21" t="inlineStr">
@@ -7422,7 +7649,7 @@
           <t>键盘盯着自己的按键，小声嘀咕：“这个怎么拼？”</t>
         </is>
       </c>
-      <c r="I129" s="43" t="inlineStr">
+      <c r="I129" s="42" t="inlineStr">
         <is>
           <t>それってどう&lt;ruby&gt;書&lt;rt&gt;か&lt;/rt&gt;&lt;/ruby&gt;くんですか？</t>
         </is>
@@ -7469,7 +7696,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>nǐ quèdìng ma？</t>
+          <t>nǐ quèdìng ma</t>
         </is>
       </c>
       <c r="H130" s="21" t="inlineStr">
@@ -7579,7 +7806,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>yǒu dàoli</t>
+          <t>yǒu dàolǐ</t>
         </is>
       </c>
       <c r="H132" s="21" t="inlineStr">
@@ -7634,7 +7861,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>ràng wǒ xiǎngxiang</t>
+          <t>ràng wǒ xiǎngxiǎng</t>
         </is>
       </c>
       <c r="H133" s="21" t="inlineStr">
@@ -7652,7 +7879,7 @@
           <t>chotto kangaesasete kudasai</t>
         </is>
       </c>
-      <c r="K133" s="44" t="inlineStr">
+      <c r="K133" s="43" t="inlineStr">
         <is>
           <t>検索バー、くるくる読み込み中。「ちょっと考えさせてください」</t>
         </is>
@@ -7744,7 +7971,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>wǒ yě bù zhīdao</t>
+          <t>wǒ yě bù zhīdào</t>
         </is>
       </c>
       <c r="H135" s="16" t="inlineStr">
@@ -7802,7 +8029,7 @@
           <t>wǒ fā xiāoxi gěi nǐ</t>
         </is>
       </c>
-      <c r="H136" s="37" t="inlineStr">
+      <c r="H136" s="36" t="inlineStr">
         <is>
           <t>萤火虫闪了两下，轻声说：“我发消息给你。”</t>
         </is>
@@ -7817,7 +8044,7 @@
           <t>messēji o okurimasu</t>
         </is>
       </c>
-      <c r="K136" s="44" t="inlineStr">
+      <c r="K136" s="43" t="inlineStr">
         <is>
           <t>ホタルがちかっ、ちかっ。「メッセージを送ります」とささやいた。</t>
         </is>
@@ -7854,7 +8081,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>néng tīngdào wǒ shuōhuà ma?</t>
+          <t>néng tīngdào wǒ shuōhuà ma</t>
         </is>
       </c>
       <c r="H137" s="21" t="inlineStr">
@@ -7872,7 +8099,7 @@
           <t>kikoemasu ka?</t>
         </is>
       </c>
-      <c r="K137" s="44" t="inlineStr">
+      <c r="K137" s="43" t="inlineStr">
         <is>
           <t>夜中の3時、火災報知器がキーン！「聞こえますか？！」</t>
         </is>
@@ -7962,9 +8189,9 @@
           <t>回头给我打个电话</t>
         </is>
       </c>
-      <c r="G139" s="46" t="inlineStr">
-        <is>
-          <t>huítóu gěi wǒ dǎ ge diànhuà</t>
+      <c r="G139" s="45" t="inlineStr">
+        <is>
+          <t>huítóu gěi wǒ dǎ gè diànhuà</t>
         </is>
       </c>
       <c r="H139" s="21" t="inlineStr">
@@ -8017,7 +8244,7 @@
           <t>看下你手机</t>
         </is>
       </c>
-      <c r="G140" s="46" t="inlineStr">
+      <c r="G140" s="45" t="inlineStr">
         <is>
           <t>kàn xià nǐ shǒujī</t>
         </is>
@@ -8074,7 +8301,7 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>kàndào wǒ fā de xiāoxi le ma?</t>
+          <t>kàndào wǒ fā de xiāoxi le ma</t>
         </is>
       </c>
       <c r="H141" s="21" t="inlineStr">
@@ -8092,7 +8319,7 @@
           <t>watashi no messēji, mite kuremashita ka?</t>
         </is>
       </c>
-      <c r="K141" s="44" t="inlineStr">
+      <c r="K141" s="43" t="inlineStr">
         <is>
           <t>びん、五回目の浜辺にぽつん。はあ……。「私のメッセージ、見てくれましたか？」</t>
         </is>
@@ -8127,9 +8354,9 @@
           <t>我在路上了</t>
         </is>
       </c>
-      <c r="G142" s="46" t="inlineStr">
-        <is>
-          <t>wǒ zài lù shang le</t>
+      <c r="G142" s="45" t="inlineStr">
+        <is>
+          <t>wǒ zài lùshang le</t>
         </is>
       </c>
       <c r="H142" s="21" t="inlineStr">
@@ -8137,7 +8364,7 @@
           <t>冰川挪了半寸，喊了一声：“我在路上了！”</t>
         </is>
       </c>
-      <c r="I142" s="43" t="inlineStr">
+      <c r="I142" s="42" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;今&lt;rt&gt;いま&lt;/rt&gt;&lt;/ruby&gt;&lt;ruby&gt;向&lt;rt&gt;む&lt;/rt&gt;&lt;/ruby&gt;かっています</t>
         </is>
@@ -8182,9 +8409,9 @@
           <t>你在哪里？</t>
         </is>
       </c>
-      <c r="G143" s="46" t="inlineStr">
-        <is>
-          <t>nǐ zài nǎlǐ?</t>
+      <c r="G143" s="45" t="inlineStr">
+        <is>
+          <t>nǐ zài nǎlǐ</t>
         </is>
       </c>
       <c r="H143" s="21" t="inlineStr">
@@ -8252,7 +8479,7 @@
           <t>あと&lt;ruby&gt;10分&lt;rt&gt;じゅっぷん&lt;/rt&gt;&lt;/ruby&gt;で&lt;ruby&gt;着&lt;rt&gt;つ&lt;/rt&gt;&lt;/ruby&gt;きます</t>
         </is>
       </c>
-      <c r="J144" s="45" t="inlineStr">
+      <c r="J144" s="44" t="inlineStr">
         <is>
           <t>ato juppun de tsukimasu</t>
         </is>
@@ -8292,9 +8519,9 @@
           <t>我能一会儿再给你打吗？</t>
         </is>
       </c>
-      <c r="G145" s="46" t="inlineStr">
-        <is>
-          <t>wǒ néng yìhuìr zài gěi nǐ dǎ ma?</t>
+      <c r="G145" s="47" t="inlineStr">
+        <is>
+          <t>wǒ néng yíhuìr zài gěi nǐ dǎ ma?</t>
         </is>
       </c>
       <c r="H145" s="21" t="inlineStr">
@@ -8307,7 +8534,7 @@
           <t>あとで&lt;ruby&gt;電話&lt;rt&gt;でんわ&lt;/rt&gt;&lt;/ruby&gt;してもいいですか？</t>
         </is>
       </c>
-      <c r="J145" s="45" t="inlineStr">
+      <c r="J145" s="44" t="inlineStr">
         <is>
           <t>ato de denwa shite mo ii desu ka?</t>
         </is>
@@ -8347,9 +8574,9 @@
           <t>给我发个短信</t>
         </is>
       </c>
-      <c r="G146" s="46" t="inlineStr">
-        <is>
-          <t>gěi wǒ fā ge duǎnxìn</t>
+      <c r="G146" s="45" t="inlineStr">
+        <is>
+          <t>gěi wǒ fā gè duǎnxìn</t>
         </is>
       </c>
       <c r="H146" s="21" t="inlineStr">
@@ -8402,9 +8629,9 @@
           <t>几点了？</t>
         </is>
       </c>
-      <c r="G147" s="46" t="inlineStr">
-        <is>
-          <t>jǐ diǎn le?</t>
+      <c r="G147" s="45" t="inlineStr">
+        <is>
+          <t>jǐ diǎn le</t>
         </is>
       </c>
       <c r="H147" s="21" t="inlineStr">
@@ -8412,7 +8639,7 @@
           <t>日晷眯着眼看云，嘀咕：“几点了？”</t>
         </is>
       </c>
-      <c r="I147" s="43" t="inlineStr">
+      <c r="I147" s="42" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;今&lt;rt&gt;いま&lt;/rt&gt;&lt;/ruby&gt;&lt;ruby&gt;何時&lt;rt&gt;なんじ&lt;/rt&gt;&lt;/ruby&gt;ですか？</t>
         </is>
@@ -8457,9 +8684,9 @@
           <t>请问几点了？</t>
         </is>
       </c>
-      <c r="G148" s="46" t="inlineStr">
-        <is>
-          <t>qǐngwèn jǐ diǎn le?</t>
+      <c r="G148" s="45" t="inlineStr">
+        <is>
+          <t>qǐngwèn jǐ diǎn le</t>
         </is>
       </c>
       <c r="H148" s="21" t="inlineStr">
@@ -8467,7 +8694,7 @@
           <t>化石睁开一只眼，含糊地问：“请问几点了？”</t>
         </is>
       </c>
-      <c r="I148" s="43" t="inlineStr">
+      <c r="I148" s="42" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;今&lt;rt&gt;いま&lt;/rt&gt;&lt;/ruby&gt;&lt;ruby&gt;何時&lt;rt&gt;なんじ&lt;/rt&gt;&lt;/ruby&gt;かわかりますか？</t>
         </is>
@@ -8512,9 +8739,9 @@
           <t>今天星期几？</t>
         </is>
       </c>
-      <c r="G149" s="46" t="inlineStr">
-        <is>
-          <t>jīntiān xīngqī jǐ?</t>
+      <c r="G149" s="45" t="inlineStr">
+        <is>
+          <t>jīntiān xīngqī jǐ</t>
         </is>
       </c>
       <c r="H149" s="21" t="inlineStr">
@@ -8527,7 +8754,7 @@
           <t>&lt;ruby&gt;今日&lt;rt&gt;きょう&lt;/rt&gt;&lt;/ruby&gt;は&lt;ruby&gt;何曜日&lt;rt&gt;なんようび&lt;/rt&gt;&lt;/ruby&gt;ですか？</t>
         </is>
       </c>
-      <c r="J149" s="45" t="inlineStr">
+      <c r="J149" s="44" t="inlineStr">
         <is>
           <t>kyō wa nan-yōbi desu ka?</t>
         </is>
@@ -8569,7 +8796,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>shénme shíhou?</t>
+          <t>shénme shíhou</t>
         </is>
       </c>
       <c r="H150" s="21" t="inlineStr">
@@ -8622,9 +8849,9 @@
           <t>几点开始？</t>
         </is>
       </c>
-      <c r="G151" s="46" t="inlineStr">
-        <is>
-          <t>jǐ diǎn kāishǐ?</t>
+      <c r="G151" s="45" t="inlineStr">
+        <is>
+          <t>jǐ diǎn kāishǐ</t>
         </is>
       </c>
       <c r="H151" s="21" t="inlineStr">
@@ -8677,6 +8904,11 @@
           <t>得多长时间？</t>
         </is>
       </c>
+      <c r="G152" s="47" t="inlineStr">
+        <is>
+          <t>děi duō cháng shíjiān?</t>
+        </is>
+      </c>
       <c r="H152" s="21" t="inlineStr">
         <is>
           <t>方便面敲着桌面哼哼：“得多长时间？”</t>
@@ -8727,6 +8959,11 @@
           <t>是不是太晚了？</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>shì búshì tài wǎn le</t>
+        </is>
+      </c>
       <c r="H153" s="21" t="inlineStr">
         <is>
           <t>牛奶盒偷瞄了眼保质期，小声问：“是不是太晚了？”</t>
@@ -8777,6 +9014,11 @@
           <t>我要迟到了</t>
         </is>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>wǒ yào chídào le</t>
+        </is>
+      </c>
       <c r="H154" s="21" t="inlineStr">
         <is>
           <t>闹钟自己睡过头了，嘀咕道：“我要迟到了。”</t>
@@ -8787,7 +9029,7 @@
           <t>&lt;ruby&gt;遅刻&lt;rt&gt;ちこく&lt;/rt&gt;&lt;/ruby&gt;しそうです</t>
         </is>
       </c>
-      <c r="J154" s="45" t="inlineStr">
+      <c r="J154" s="44" t="inlineStr">
         <is>
           <t>chikoku shisō desu</t>
         </is>
@@ -8827,12 +9069,17 @@
           <t>能改个时间吗？</t>
         </is>
       </c>
+      <c r="G155" s="45" t="inlineStr">
+        <is>
+          <t>néng gǎi gè shíjiān ma</t>
+        </is>
+      </c>
       <c r="H155" s="21" t="inlineStr">
         <is>
           <t>牙医椅一看见你进来就喊：“能改个时间吗？”</t>
         </is>
       </c>
-      <c r="I155" s="42" t="inlineStr">
+      <c r="I155" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;予約&lt;rt&gt;よやく&lt;/rt&gt;&lt;/ruby&gt;を&lt;ruby&gt;変更&lt;rt&gt;へんこう&lt;/rt&gt;&lt;/ruby&gt;できますか？</t>
         </is>
@@ -8877,6 +9124,11 @@
           <t>我晚点回复你</t>
         </is>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>wǒ wǎndiǎn huífù nǐ</t>
+        </is>
+      </c>
       <c r="H156" s="21" t="inlineStr">
         <is>
           <t>悠悠球从桌上滚下去，喊道：“我晚点回复你！”</t>
@@ -8892,7 +9144,7 @@
           <t>ato de renraku shimasu</t>
         </is>
       </c>
-      <c r="K156" s="44" t="inlineStr">
+      <c r="K156" s="43" t="inlineStr">
         <is>
           <t>ヨーヨー、テーブルからころん。「あとで連絡します！」とさけぶ。</t>
         </is>
@@ -8927,6 +9179,11 @@
           <t>我先看看安排</t>
         </is>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>wǒ xiān kànkan ānpái</t>
+        </is>
+      </c>
       <c r="H157" s="22" t="inlineStr">
         <is>
           <t>日历哗啦啦翻着自己：“我先看看安排。”</t>
@@ -8977,7 +9234,12 @@
           <t>我在弄了</t>
         </is>
       </c>
-      <c r="H158" s="38" t="inlineStr">
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>wǒ zài nòng le</t>
+        </is>
+      </c>
+      <c r="H158" s="37" t="inlineStr">
         <is>
           <t>面团鼓了鼓肚子说：“我在弄了。”</t>
         </is>
@@ -8992,7 +9254,7 @@
           <t>ima yatte imasu</t>
         </is>
       </c>
-      <c r="K158" s="38" t="inlineStr">
+      <c r="K158" s="37" t="inlineStr">
         <is>
           <t>パン生地、ぷくっとふくらんで、「今やっています」</t>
         </is>
@@ -9027,6 +9289,11 @@
           <t>你能帮我一下吗？</t>
         </is>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>nǐ néng bāng wǒ yīxià ma</t>
+        </is>
+      </c>
       <c r="H159" s="21" t="inlineStr">
         <is>
           <t>拉链卡在半路，哼唧道：“你能帮我一下吗？”</t>
@@ -9077,6 +9344,11 @@
           <t>我没搞懂</t>
         </is>
       </c>
+      <c r="G160" s="45" t="inlineStr">
+        <is>
+          <t>wǒ méi gǎodǒng</t>
+        </is>
+      </c>
       <c r="H160" s="21" t="inlineStr">
         <is>
           <t>数学课本翻着自己，嘟囔道：“我没搞懂。”</t>
@@ -9127,6 +9399,11 @@
           <t>能带我从头过一遍吗？</t>
         </is>
       </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>néng dài wǒ cóngtóu guò yībiàn ma</t>
+        </is>
+      </c>
       <c r="H161" s="22" t="inlineStr">
         <is>
           <t>迷宫盯着自己弯弯绕绕的路：“能带我从头过一遍吗？”</t>
@@ -9182,7 +9459,7 @@
           <t>jiézhǐ rìqī shì shénme shíhou？</t>
         </is>
       </c>
-      <c r="H162" s="37" t="inlineStr">
+      <c r="H162" s="36" t="inlineStr">
         <is>
           <t>香蕉看看身上的褐色小斑点，伤心地问：“截止日期是什么时候？”</t>
         </is>
@@ -9232,9 +9509,9 @@
           <t>我这就发过去</t>
         </is>
       </c>
-      <c r="G163" s="46" t="inlineStr">
-        <is>
-          <t>wǒ zhè jiù fā guòqu</t>
+      <c r="G163" s="45" t="inlineStr">
+        <is>
+          <t>wǒ zhè jiù fā guòqù</t>
         </is>
       </c>
       <c r="H163" s="21" t="inlineStr">
@@ -9242,7 +9519,7 @@
           <t>弹弓装上小石子，笑嘻嘻地说：“我这就发过去！”</t>
         </is>
       </c>
-      <c r="I163" s="42" t="inlineStr">
+      <c r="I163" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;今&lt;rt&gt;いま&lt;/rt&gt;&lt;/ruby&gt;すぐ&lt;ruby&gt;送&lt;rt&gt;おく&lt;/rt&gt;&lt;/ruby&gt;ります</t>
         </is>
@@ -9287,9 +9564,9 @@
           <t>我能问你个事吗？</t>
         </is>
       </c>
-      <c r="G164" s="46" t="inlineStr">
-        <is>
-          <t>wǒ néng wèn nǐ ge shì ma?</t>
+      <c r="G164" s="45" t="inlineStr">
+        <is>
+          <t>wǒ néng wèn nǐ gè shì ma？</t>
         </is>
       </c>
       <c r="H164" s="21" t="inlineStr">
@@ -9307,7 +9584,7 @@
           <t>chotto kiite mo ii desu ka?</t>
         </is>
       </c>
-      <c r="K164" s="44" t="inlineStr">
+      <c r="K164" s="43" t="inlineStr">
         <is>
           <t>フォーチュンクッキーがパキッと割れて、こっそり「ちょっと聞いてもいいですか？」</t>
         </is>
@@ -9344,10 +9621,10 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>zhèyàng jiǎng qīngchu le ma？</t>
-        </is>
-      </c>
-      <c r="H165" s="37" t="inlineStr">
+          <t>zhèyàng jiǎng qīngchǔ le ma？</t>
+        </is>
+      </c>
+      <c r="H165" s="36" t="inlineStr">
         <is>
           <t>抽象画歪了歪身子：“这样讲清楚了吗？”</t>
         </is>
@@ -9362,7 +9639,7 @@
           <t>tsutawarimashita ka?</t>
         </is>
       </c>
-      <c r="K165" s="44" t="inlineStr">
+      <c r="K165" s="43" t="inlineStr">
         <is>
           <t>抽象画はこてんと首をかしげて、「伝わりましたか？」</t>
         </is>
@@ -9454,7 +9731,7 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>wǒmen xiūxi yíxià ba</t>
+          <t>wǒmen xiūxi yīxià ba</t>
         </is>
       </c>
       <c r="H167" s="21" t="inlineStr">
@@ -9672,9 +9949,9 @@
           <t>我来洗碗</t>
         </is>
       </c>
-      <c r="G171" s="46" t="inlineStr">
-        <is>
-          <t>wǒ lái xǐ wǎn</t>
+      <c r="G171" s="45" t="inlineStr">
+        <is>
+          <t>wǒ lái xǐwǎn</t>
         </is>
       </c>
       <c r="H171" s="21" t="inlineStr">
@@ -9729,7 +10006,7 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>Nǐ néng guān xià dēng ma？</t>
+          <t>nǐ néng guān xià dēng ma</t>
         </is>
       </c>
       <c r="H172" s="22" t="inlineStr">
@@ -9782,9 +10059,9 @@
           <t>你看到我的钥匙了吗？</t>
         </is>
       </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>Nǐ kàndào wǒ de yàoshi le ma？</t>
+      <c r="G173" s="47" t="inlineStr">
+        <is>
+          <t>nǐ kàndào wǒ de yàoshi le ma?</t>
         </is>
       </c>
       <c r="H173" s="21" t="inlineStr">
@@ -9802,7 +10079,7 @@
           <t>kagi o mikakemasen deshita ka?</t>
         </is>
       </c>
-      <c r="K173" s="44" t="inlineStr">
+      <c r="K173" s="43" t="inlineStr">
         <is>
           <t>ドアの鍵穴は毎朝はあっとため息。「鍵を見かけませんでしたか？」</t>
         </is>
@@ -9839,7 +10116,7 @@
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Wǒ děi xǐ yīfu le</t>
+          <t>wǒ děi xǐ yīfu le</t>
         </is>
       </c>
       <c r="H174" s="21" t="inlineStr">
@@ -9894,7 +10171,7 @@
       </c>
       <c r="G175" t="inlineStr">
         <is>
-          <t>Wèishēngzhǐ yòngwán le</t>
+          <t>wèishēngzhǐ yòngwán le</t>
         </is>
       </c>
       <c r="H175" s="21" t="inlineStr">
@@ -9912,7 +10189,7 @@
           <t>toirettopēpā ga kirete imasu</t>
         </is>
       </c>
-      <c r="K175" s="44" t="inlineStr">
+      <c r="K175" s="43" t="inlineStr">
         <is>
           <t>トイレットペーパーホルダー、下を見てしょんぼり。「トイレットペーパーが切れています！」</t>
         </is>
@@ -9947,9 +10224,9 @@
           <t>能把那个捡起来吗？</t>
         </is>
       </c>
-      <c r="G176" s="46" t="inlineStr">
-        <is>
-          <t>néng bǎ nàge jiǎn qilai ma?</t>
+      <c r="G176" s="45" t="inlineStr">
+        <is>
+          <t>néng bǎ nàge jiǎn qǐlái ma</t>
         </is>
       </c>
       <c r="H176" s="21" t="inlineStr">
@@ -9967,7 +10244,7 @@
           <t>sore, hirotte kuremasu ka?</t>
         </is>
       </c>
-      <c r="K176" s="44" t="inlineStr">
+      <c r="K176" s="43" t="inlineStr">
         <is>
           <t>お掃除ロボット、靴下にごつん。「それ、拾ってくれますか？」</t>
         </is>
@@ -10002,9 +10279,9 @@
           <t>我今天晚点到家</t>
         </is>
       </c>
-      <c r="G177" s="46" t="inlineStr">
-        <is>
-          <t>wǒ jīntiān wǎndiǎn dào jiā</t>
+      <c r="G177" s="45" t="inlineStr">
+        <is>
+          <t>wǒ jīntiān wǎn diǎn dào jiā</t>
         </is>
       </c>
       <c r="H177" s="21" t="inlineStr">
@@ -10059,7 +10336,7 @@
       </c>
       <c r="G178" t="inlineStr">
         <is>
-          <t>Bié wàng le dài sǎn</t>
+          <t>bié wàng le dài sǎn</t>
         </is>
       </c>
       <c r="H178" s="21" t="inlineStr">
@@ -10077,7 +10354,7 @@
           <t>kasa o owasurenaku</t>
         </is>
       </c>
-      <c r="K178" s="44" t="inlineStr">
+      <c r="K178" s="43" t="inlineStr">
         <is>
           <t>雲がひょっこり顔を出して、「傘をお忘れなく！」</t>
         </is>
@@ -10112,12 +10389,12 @@
           <t>七点叫我起床</t>
         </is>
       </c>
-      <c r="G179" s="46" t="inlineStr">
+      <c r="G179" s="45" t="inlineStr">
         <is>
           <t>qī diǎn jiào wǒ qǐchuáng</t>
         </is>
       </c>
-      <c r="H179" s="37" t="inlineStr">
+      <c r="H179" s="36" t="inlineStr">
         <is>
           <t>拖鞋小声说：“七点叫我起床，早上还要去散步呢。”</t>
         </is>
@@ -10169,7 +10446,7 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Wǒ shuìbuzháo</t>
+          <t>wǒ shuì bu zháo</t>
         </is>
       </c>
       <c r="H180" s="16" t="inlineStr">
@@ -10187,7 +10464,7 @@
           <t>nemurenai</t>
         </is>
       </c>
-      <c r="K180" s="44" t="inlineStr">
+      <c r="K180" s="43" t="inlineStr">
         <is>
           <t>ベッドは天井をじっと見つめて、はあ。「眠れない……」</t>
         </is>
@@ -10224,7 +10501,7 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>Wǒ qù shuì le</t>
+          <t>wǒ qù shuì le</t>
         </is>
       </c>
       <c r="H181" s="21" t="inlineStr">
@@ -10297,7 +10574,7 @@
           <t>gohan desu yo</t>
         </is>
       </c>
-      <c r="K182" s="44" t="inlineStr">
+      <c r="K182" s="43" t="inlineStr">
         <is>
           <t>ローストチキンがオーブンからぴょこん。「ごはんですよ！」</t>
         </is>
@@ -10497,17 +10774,17 @@
           <t>算我一个</t>
         </is>
       </c>
-      <c r="G186" s="46" t="inlineStr">
-        <is>
-          <t>suàn wǒ yíge</t>
-        </is>
-      </c>
-      <c r="H186" s="37" t="inlineStr">
+      <c r="G186" s="47" t="inlineStr">
+        <is>
+          <t>suàn wǒ yí gè</t>
+        </is>
+      </c>
+      <c r="H186" s="36" t="inlineStr">
         <is>
           <t>爆米花一听到“今晚看电影”，就大喊：“算我一个！”</t>
         </is>
       </c>
-      <c r="I186" s="43" t="inlineStr">
+      <c r="I186" s="42" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;私&lt;rt&gt;わたし&lt;/rt&gt;&lt;/ruby&gt;も&lt;ruby&gt;入&lt;rt&gt;い&lt;/rt&gt;&lt;/ruby&gt;れてください</t>
         </is>
@@ -10517,7 +10794,7 @@
           <t>watashi mo irete kudasai</t>
         </is>
       </c>
-      <c r="K186" s="44" t="inlineStr">
+      <c r="K186" s="43" t="inlineStr">
         <is>
           <t>「今夜は映画だよ」と聞いて、ポップコーンがぱんっ。「私も入れてください！」</t>
         </is>
@@ -10552,7 +10829,7 @@
           <t>别算上我</t>
         </is>
       </c>
-      <c r="G187" s="46" t="inlineStr">
+      <c r="G187" s="45" t="inlineStr">
         <is>
           <t>bié suàn shàng wǒ</t>
         </is>
@@ -10617,7 +10894,7 @@
           <t>门挡把自己一脚踢开，喊道：“走吧！”</t>
         </is>
       </c>
-      <c r="I188" s="42" t="inlineStr">
+      <c r="I188" s="41" t="inlineStr">
         <is>
           <t>&lt;ruby&gt;行&lt;rt&gt;い&lt;/rt&gt;&lt;/ruby&gt;きましょう</t>
         </is>
@@ -10627,7 +10904,7 @@
           <t>ikimashō</t>
         </is>
       </c>
-      <c r="K188" s="44" t="inlineStr">
+      <c r="K188" s="43" t="inlineStr">
         <is>
           <t>ドアストッパーは自分をぽーんと蹴飛ばして、「行きましょう！」</t>
         </is>
@@ -10717,12 +10994,12 @@
           <t>等一下</t>
         </is>
       </c>
-      <c r="G190" t="inlineStr">
+      <c r="G190" s="47" t="inlineStr">
         <is>
           <t>děng yíxià</t>
         </is>
       </c>
-      <c r="H190" s="37" t="inlineStr">
+      <c r="H190" s="36" t="inlineStr">
         <is>
           <t>进度条跳到99%，叮地一声说：“等一下。”</t>
         </is>
@@ -10772,9 +11049,9 @@
           <t>算了算了</t>
         </is>
       </c>
-      <c r="G191" s="46" t="inlineStr">
-        <is>
-          <t>suàn le suàn le</t>
+      <c r="G191" s="45" t="inlineStr">
+        <is>
+          <t>suànle suànle</t>
         </is>
       </c>
       <c r="H191" s="16" t="inlineStr">
@@ -10782,12 +11059,12 @@
           <t>金属探测器哔了一声，然后叹了口气：“算了算了。”</t>
         </is>
       </c>
-      <c r="I191" s="42" t="inlineStr">
+      <c r="I191" s="41" t="inlineStr">
         <is>
           <t>なんでもないです</t>
         </is>
       </c>
-      <c r="J191" s="45" t="inlineStr">
+      <c r="J191" s="44" t="inlineStr">
         <is>
           <t>nan demo nai desu</t>
         </is>
@@ -10827,7 +11104,7 @@
           <t>没什么大不了的</t>
         </is>
       </c>
-      <c r="G192" s="46" t="inlineStr">
+      <c r="G192" s="47" t="inlineStr">
         <is>
           <t>méi shénme dàbuliǎo de</t>
         </is>
@@ -10939,7 +11216,7 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>wǒ wánquán bù zhīdao</t>
+          <t>wǒ wánquán bù zhīdào</t>
         </is>
       </c>
       <c r="H194" s="16" t="inlineStr">
@@ -11049,7 +11326,7 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>shuō shíhuà，wǒ gēnběn bú zàihu</t>
+          <t>shuō shíhuà, wǒ gēnběn bù zàihu</t>
         </is>
       </c>
       <c r="H196" s="21" t="inlineStr">
@@ -11104,7 +11381,7 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>zhēn de jiǎ de？</t>
+          <t>zhēnde jiǎde?</t>
         </is>
       </c>
       <c r="H197" s="21" t="inlineStr">
@@ -11153,7 +11430,7 @@
           <t>你那边信号不好</t>
         </is>
       </c>
-      <c r="G198" s="47" t="inlineStr">
+      <c r="G198" s="46" t="inlineStr">
         <is>
           <t>nǐ nàbiān xìnhào bù hǎo</t>
         </is>
@@ -11187,7 +11464,7 @@
       </c>
       <c r="G199" s="1" t="inlineStr">
         <is>
-          <t>zhīdao le</t>
+          <t>zhīdào le</t>
         </is>
       </c>
       <c r="H199" s="32" t="n"/>

</xml_diff>

<commit_message>
Data sync: row 14 IPA filled in, +1 phrase (196 total), sw v57
User filled in 英语音标 for "How are you today?" so it now passes
completeness check and ships. Rows 198/199 still incomplete by design
(holding off per user).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/update_data_folder/PhraseList.xlsx
+++ b/update_data_folder/PhraseList.xlsx
@@ -1308,7 +1308,11 @@
       <c r="D14" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="13" t="n"/>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>/haʊ ɑːr juː təˈdeɪ/</t>
+        </is>
+      </c>
       <c r="F14" s="34" t="inlineStr">
         <is>
           <t>你今天怎么样？</t>
@@ -11457,6 +11461,11 @@
       <c r="B199" s="13" t="n"/>
       <c r="C199" s="13" t="n"/>
       <c r="D199" s="13" t="n"/>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>/ɡɑːt ɪt/</t>
+        </is>
+      </c>
       <c r="F199" s="34" t="inlineStr">
         <is>
           <t>知道了</t>

</xml_diff>